<commit_message>
fix: set UAT environment in Susana incident example
</commit_message>
<xml_diff>
--- a/docs/excel/incidentes-susana-antilaf.xlsx
+++ b/docs/excel/incidentes-susana-antilaf.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incidentes" sheetId="1" r:id="Rd1a843056bf0411b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="R8a6e4fb50c0646db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Incidentes" sheetId="1" r:id="Rd730c8af504b4c0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instrucciones" sheetId="2" r:id="Rc45c6dfcdf214f5a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -413,7 +413,9 @@
       <x:c r="C2" s="3" t="str">
         <x:v>Compraqui tarjetas: Nuevo por inconsistencia queda asociado al carro, pero no muestra todos los valores.</x:v>
       </x:c>
-      <x:c r="D2" s="9" t="str"/>
+      <x:c r="D2" s="9" t="str">
+        <x:v>UAT</x:v>
+      </x:c>
       <x:c r="E2" s="9" t="str"/>
       <x:c r="F2" s="3" t="str">
         <x:v>Susana Antilaf</x:v>
@@ -444,7 +446,9 @@
       <x:c r="C3" s="3" t="str">
         <x:v>Compra Aquí Tarjetas, pago faltante no se visualiza en reporte de pagos ventas.</x:v>
       </x:c>
-      <x:c r="D3" s="9" t="str"/>
+      <x:c r="D3" s="9" t="str">
+        <x:v>UAT</x:v>
+      </x:c>
       <x:c r="E3" s="9" t="str"/>
       <x:c r="F3" s="3" t="str">
         <x:v>Susana Antilaf</x:v>
@@ -475,7 +479,9 @@
       <x:c r="C4" s="3" t="str">
         <x:v>Pagos faltantes no queda asociado al carro, lo que genera reporte con datos vacíos.</x:v>
       </x:c>
-      <x:c r="D4" s="9" t="str"/>
+      <x:c r="D4" s="9" t="str">
+        <x:v>UAT</x:v>
+      </x:c>
       <x:c r="E4" s="9" t="str"/>
       <x:c r="F4" s="3" t="str">
         <x:v>Susana Antilaf</x:v>
@@ -506,7 +512,9 @@
       <x:c r="C5" s="3" t="str">
         <x:v>Compraqui QR/login: Al procesar el archivo BIL, finaliza la tarea correctamente, pero no hace nada.</x:v>
       </x:c>
-      <x:c r="D5" s="9" t="str"/>
+      <x:c r="D5" s="9" t="str">
+        <x:v>UAT</x:v>
+      </x:c>
       <x:c r="E5" s="9" t="str"/>
       <x:c r="F5" s="3" t="str">
         <x:v>Susana Antilaf</x:v>
@@ -537,7 +545,9 @@
       <x:c r="C6" s="3" t="str">
         <x:v>Novedades, pagos faltantes el mensaje de notificación tiene campos en blanco y no detalla los ítems del carro.</x:v>
       </x:c>
-      <x:c r="D6" s="9" t="str"/>
+      <x:c r="D6" s="9" t="str">
+        <x:v>UAT</x:v>
+      </x:c>
       <x:c r="E6" s="9" t="str"/>
       <x:c r="F6" s="3" t="str">
         <x:v>Susana Antilaf</x:v>
@@ -568,7 +578,9 @@
       <x:c r="C7" s="3" t="str">
         <x:v>Novedades, pagos sobrantes: el mensaje de notificación no es igual al mensaje de notificación original.</x:v>
       </x:c>
-      <x:c r="D7" s="9" t="str"/>
+      <x:c r="D7" s="9" t="str">
+        <x:v>UAT</x:v>
+      </x:c>
       <x:c r="E7" s="9" t="str"/>
       <x:c r="F7" s="3" t="str">
         <x:v>Susana Antilaf</x:v>
@@ -602,7 +614,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R1a463e43813b49c9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R110598f09ba94a1a"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -652,7 +664,7 @@
         <x:v>Ambiente</x:v>
       </x:c>
       <x:c r="B5" s="11" t="str">
-        <x:v>DESA, CERT, UAT o PROD. El reporte de Susana no indica el ambiente: confírmalo antes de cargar.</x:v>
+        <x:v>UAT, indicado por el usuario para las seis incidencias de este reporte.</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="48" customHeight="1">
@@ -756,7 +768,7 @@
         <x:v>Campos por completar</x:v>
       </x:c>
       <x:c r="B18" s="11" t="str">
-        <x:v>El proyecto, el ambiente, las prioridades y los responsables por email no aparecen en el reporte. Proyecto y ambiente se eligen al subir; responsables y prioridad pueden completarse después.</x:v>
+        <x:v>El proyecto, las prioridades y los responsables por email no aparecen en el reporte. Selecciona el proyecto al subir; el ambiente UAT ya está completado.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>